<commit_message>
spm-25 and test cases
</commit_message>
<xml_diff>
--- a/docs/test-cases/SPM-24_Test_Cases.xlsx
+++ b/docs/test-cases/SPM-24_Test_Cases.xlsx
@@ -25,6 +25,7 @@
     <sheet name="TC15" sheetId="17" state="visible" r:id="rId17"/>
     <sheet name="TC16" sheetId="18" state="visible" r:id="rId18"/>
     <sheet name="TC17" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet name="TC18" sheetId="20" state="visible" r:id="rId20"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -464,7 +465,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F30"/>
+  <dimension ref="A1:F31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -920,7 +921,7 @@
       </c>
       <c r="C16" s="11" t="inlineStr">
         <is>
-          <t>Replacing equipment with the same item twice in a draft edit is rejected</t>
+          <t>An equipment item already chosen in one row is not offered again in another row</t>
         </is>
       </c>
       <c r="D16" s="11" t="inlineStr">
@@ -930,7 +931,7 @@
       </c>
       <c r="E16" s="11" t="inlineStr">
         <is>
-          <t>Negative</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="F16" s="11" t="inlineStr">
@@ -947,27 +948,27 @@
       </c>
       <c r="B17" s="11" t="inlineStr">
         <is>
-          <t>SPM-24-TC14</t>
+          <t>SPM-24-TC13b</t>
         </is>
       </c>
       <c r="C17" s="11" t="inlineStr">
         <is>
-          <t>A complete draft can be submitted and leaves draft status</t>
+          <t>"Add equipment" is disabled once every catalogue item is already in the request</t>
         </is>
       </c>
       <c r="D17" s="11" t="inlineStr">
         <is>
-          <t>AC1, AC5</t>
+          <t>AC4</t>
         </is>
       </c>
       <c r="E17" s="11" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>Boundary</t>
         </is>
       </c>
       <c r="F17" s="11" t="inlineStr">
         <is>
-          <t>Acceptance Criteria</t>
+          <t>Code</t>
         </is>
       </c>
     </row>
@@ -979,27 +980,27 @@
       </c>
       <c r="B18" s="11" t="inlineStr">
         <is>
-          <t>SPM-24-TC15</t>
+          <t>SPM-24-TC14</t>
         </is>
       </c>
       <c r="C18" s="11" t="inlineStr">
         <is>
-          <t>An incomplete draft cannot be submitted from its edit page</t>
+          <t>A complete draft can be submitted and leaves draft status</t>
         </is>
       </c>
       <c r="D18" s="11" t="inlineStr">
         <is>
-          <t>AC5</t>
+          <t>AC1, AC5</t>
         </is>
       </c>
       <c r="E18" s="11" t="inlineStr">
         <is>
-          <t>Negative</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="F18" s="11" t="inlineStr">
         <is>
-          <t>Code</t>
+          <t>Acceptance Criteria</t>
         </is>
       </c>
     </row>
@@ -1011,12 +1012,12 @@
       </c>
       <c r="B19" s="11" t="inlineStr">
         <is>
-          <t>SPM-24-TC16</t>
+          <t>SPM-24-TC15</t>
         </is>
       </c>
       <c r="C19" s="11" t="inlineStr">
         <is>
-          <t>A draft never appears in the Submitted section of the owner's own events page</t>
+          <t>An incomplete draft cannot be submitted from its edit page</t>
         </is>
       </c>
       <c r="D19" s="11" t="inlineStr">
@@ -1026,7 +1027,7 @@
       </c>
       <c r="E19" s="11" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="F19" s="11" t="inlineStr">
@@ -1043,64 +1044,96 @@
       </c>
       <c r="B20" s="11" t="inlineStr">
         <is>
+          <t>SPM-24-TC16</t>
+        </is>
+      </c>
+      <c r="C20" s="11" t="inlineStr">
+        <is>
+          <t>A draft never appears in the Submitted section of the owner's own events page</t>
+        </is>
+      </c>
+      <c r="D20" s="11" t="inlineStr">
+        <is>
+          <t>AC5</t>
+        </is>
+      </c>
+      <c r="E20" s="11" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="F20" s="11" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="10" t="inlineStr">
+        <is>
+          <t>TC18</t>
+        </is>
+      </c>
+      <c r="B21" s="11" t="inlineStr">
+        <is>
           <t>SPM-24-TC17</t>
         </is>
       </c>
-      <c r="C20" s="11" t="inlineStr">
+      <c r="C21" s="11" t="inlineStr">
         <is>
           <t>A non-organiser role never sees another user's draft in the events list</t>
         </is>
       </c>
-      <c r="D20" s="11" t="inlineStr">
+      <c r="D21" s="11" t="inlineStr">
         <is>
           <t>AC3, AC5</t>
         </is>
       </c>
-      <c r="E20" s="11" t="inlineStr">
+      <c r="E21" s="11" t="inlineStr">
         <is>
           <t>Positive</t>
         </is>
       </c>
-      <c r="F20" s="11" t="inlineStr">
+      <c r="F21" s="11" t="inlineStr">
         <is>
           <t>Code</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="7" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="7" t="inlineStr">
         <is>
           <t>AC</t>
         </is>
       </c>
-      <c r="B23" s="7" t="inlineStr">
+      <c r="B24" s="7" t="inlineStr">
         <is>
           <t>Acceptance Criterion</t>
-        </is>
-      </c>
-      <c r="C23" s="8" t="n"/>
-      <c r="D23" s="9" t="n"/>
-      <c r="E23" s="7" t="inlineStr">
-        <is>
-          <t>Covered by</t>
-        </is>
-      </c>
-      <c r="F23" s="9" t="n"/>
-    </row>
-    <row r="24" ht="58" customHeight="1">
-      <c r="A24" s="11" t="inlineStr">
-        <is>
-          <t>AC1</t>
-        </is>
-      </c>
-      <c r="B24" s="11" t="inlineStr">
-        <is>
-          <t>Given I have entered some event information, when I select "Save Draft", then the request is saved.</t>
         </is>
       </c>
       <c r="C24" s="8" t="n"/>
       <c r="D24" s="9" t="n"/>
-      <c r="E24" s="11" t="inlineStr">
+      <c r="E24" s="7" t="inlineStr">
+        <is>
+          <t>Covered by</t>
+        </is>
+      </c>
+      <c r="F24" s="9" t="n"/>
+    </row>
+    <row r="25" ht="58" customHeight="1">
+      <c r="A25" s="11" t="inlineStr">
+        <is>
+          <t>AC1</t>
+        </is>
+      </c>
+      <c r="B25" s="11" t="inlineStr">
+        <is>
+          <t>Given I have entered some event information, when I select "Save Draft", then the request is saved.</t>
+        </is>
+      </c>
+      <c r="C25" s="8" t="n"/>
+      <c r="D25" s="9" t="n"/>
+      <c r="E25" s="11" t="inlineStr">
         <is>
           <t>SPM-24-TC01
 SPM-24-TC02
@@ -1108,43 +1141,43 @@
 SPM-24-TC14</t>
         </is>
       </c>
-      <c r="F24" s="9" t="n"/>
-    </row>
-    <row r="25" ht="31" customHeight="1">
-      <c r="A25" s="11" t="inlineStr">
+      <c r="F25" s="9" t="n"/>
+    </row>
+    <row r="26" ht="31" customHeight="1">
+      <c r="A26" s="11" t="inlineStr">
         <is>
           <t>AC2</t>
         </is>
       </c>
-      <c r="B25" s="11" t="inlineStr">
+      <c r="B26" s="11" t="inlineStr">
         <is>
           <t>A saved draft is clearly identified as a draft.</t>
-        </is>
-      </c>
-      <c r="C25" s="8" t="n"/>
-      <c r="D25" s="9" t="n"/>
-      <c r="E25" s="11" t="inlineStr">
-        <is>
-          <t>SPM-24-TC04
-SPM-24-TC05</t>
-        </is>
-      </c>
-      <c r="F25" s="9" t="n"/>
-    </row>
-    <row r="26" ht="58" customHeight="1">
-      <c r="A26" s="11" t="inlineStr">
-        <is>
-          <t>AC3</t>
-        </is>
-      </c>
-      <c r="B26" s="11" t="inlineStr">
-        <is>
-          <t>I can leave the system and return to the draft later.</t>
         </is>
       </c>
       <c r="C26" s="8" t="n"/>
       <c r="D26" s="9" t="n"/>
       <c r="E26" s="11" t="inlineStr">
+        <is>
+          <t>SPM-24-TC04
+SPM-24-TC05</t>
+        </is>
+      </c>
+      <c r="F26" s="9" t="n"/>
+    </row>
+    <row r="27" ht="58" customHeight="1">
+      <c r="A27" s="11" t="inlineStr">
+        <is>
+          <t>AC3</t>
+        </is>
+      </c>
+      <c r="B27" s="11" t="inlineStr">
+        <is>
+          <t>I can leave the system and return to the draft later.</t>
+        </is>
+      </c>
+      <c r="C27" s="8" t="n"/>
+      <c r="D27" s="9" t="n"/>
+      <c r="E27" s="11" t="inlineStr">
         <is>
           <t>SPM-24-TC06
 SPM-24-TC07
@@ -1152,46 +1185,47 @@
 SPM-24-TC17</t>
         </is>
       </c>
-      <c r="F26" s="9" t="n"/>
-    </row>
-    <row r="27" ht="71.5" customHeight="1">
-      <c r="A27" s="11" t="inlineStr">
+      <c r="F27" s="9" t="n"/>
+    </row>
+    <row r="28" ht="85" customHeight="1">
+      <c r="A28" s="11" t="inlineStr">
         <is>
           <t>AC4</t>
         </is>
       </c>
-      <c r="B27" s="11" t="inlineStr">
+      <c r="B28" s="11" t="inlineStr">
         <is>
           <t>I can edit the information in the draft.</t>
         </is>
       </c>
-      <c r="C27" s="8" t="n"/>
-      <c r="D27" s="9" t="n"/>
-      <c r="E27" s="11" t="inlineStr">
+      <c r="C28" s="8" t="n"/>
+      <c r="D28" s="9" t="n"/>
+      <c r="E28" s="11" t="inlineStr">
         <is>
           <t>SPM-24-TC09
 SPM-24-TC10
 SPM-24-TC11
 SPM-24-TC12
-SPM-24-TC13</t>
-        </is>
-      </c>
-      <c r="F27" s="9" t="n"/>
-    </row>
-    <row r="28" ht="71.5" customHeight="1">
-      <c r="A28" s="11" t="inlineStr">
+SPM-24-TC13
+SPM-24-TC13b</t>
+        </is>
+      </c>
+      <c r="F28" s="9" t="n"/>
+    </row>
+    <row r="29" ht="71.5" customHeight="1">
+      <c r="A29" s="11" t="inlineStr">
         <is>
           <t>AC5</t>
         </is>
       </c>
-      <c r="B28" s="11" t="inlineStr">
+      <c r="B29" s="11" t="inlineStr">
         <is>
           <t>A draft is not treated as a submitted event request.</t>
         </is>
       </c>
-      <c r="C28" s="8" t="n"/>
-      <c r="D28" s="9" t="n"/>
-      <c r="E28" s="11" t="inlineStr">
+      <c r="C29" s="8" t="n"/>
+      <c r="D29" s="9" t="n"/>
+      <c r="E29" s="11" t="inlineStr">
         <is>
           <t>SPM-24-TC12
 SPM-24-TC14
@@ -1200,15 +1234,15 @@
 SPM-24-TC17</t>
         </is>
       </c>
-      <c r="F28" s="9" t="n"/>
-    </row>
-    <row r="30" ht="152.5" customHeight="1">
-      <c r="A30" s="7" t="inlineStr">
+      <c r="F29" s="9" t="n"/>
+    </row>
+    <row r="31" ht="152.5" customHeight="1">
+      <c r="A31" s="7" t="inlineStr">
         <is>
           <t>Code reviewed</t>
         </is>
       </c>
-      <c r="B30" s="11" t="inlineStr">
+      <c r="B31" s="11" t="inlineStr">
         <is>
           <t>src/lib/validation.ts
 src/lib/eventForm.ts
@@ -1223,24 +1257,24 @@
 prisma/seed.ts</t>
         </is>
       </c>
-      <c r="C30" s="8" t="n"/>
-      <c r="D30" s="8" t="n"/>
-      <c r="E30" s="8" t="n"/>
-      <c r="F30" s="9" t="n"/>
+      <c r="C31" s="8" t="n"/>
+      <c r="D31" s="8" t="n"/>
+      <c r="E31" s="8" t="n"/>
+      <c r="F31" s="9" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="14">
-    <mergeCell ref="B30:F30"/>
     <mergeCell ref="B28:D28"/>
-    <mergeCell ref="B23:D23"/>
+    <mergeCell ref="E29:F29"/>
     <mergeCell ref="E24:F24"/>
     <mergeCell ref="E25:F25"/>
     <mergeCell ref="B26:D26"/>
     <mergeCell ref="B27:D27"/>
-    <mergeCell ref="E23:F23"/>
     <mergeCell ref="E27:F27"/>
     <mergeCell ref="E28:F28"/>
+    <mergeCell ref="B31:F31"/>
     <mergeCell ref="B1:F1"/>
+    <mergeCell ref="B29:D29"/>
     <mergeCell ref="E26:F26"/>
     <mergeCell ref="B25:D25"/>
     <mergeCell ref="B24:D24"/>
@@ -1263,6 +1297,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A18" r:id="rId15"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A19" r:id="rId16"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A20" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A21" r:id="rId18"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2100,7 +2135,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="17.5" customHeight="1">
+    <row r="3" ht="31" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
@@ -2108,11 +2143,11 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>The draft from TC09 already has Starts at and Ends at saved.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="85" customHeight="1">
+          <t>The draft from TC09 already has Starts at and Ends at saved. The equipment catalogue has at least two active items.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="71.5" customHeight="1">
       <c r="A4" s="12" t="inlineStr">
         <is>
           <t>Test Steps</t>
@@ -2121,13 +2156,13 @@
       <c r="B4" s="13" t="inlineStr">
         <is>
           <t>1. Open the draft's "Edit draft" page
-2. Add an equipment row, choose "4K Portable Projector", quantity 1
-3. Add a second equipment row, choose "4K Portable Projector" again, quantity 2
-4. Click "Save draft"</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="31" customHeight="1">
+2. Click "Add equipment" and choose "4K Portable Projector" in the first row
+3. Click "Add equipment" again to add a second row
+4. Open the second row's equipment dropdown</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="17.5" customHeight="1">
       <c r="A5" s="12" t="inlineStr">
         <is>
           <t>Test Data</t>
@@ -2135,7 +2170,7 @@
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>Equipment: "4K Portable Projector" chosen in two separate rows</t>
+          <t>First row: 4K Portable Projector</t>
         </is>
       </c>
     </row>
@@ -2147,7 +2182,7 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>The page does not move on. A message "Each item can only be requested once — change the quantity instead of adding a second row." appears above the equipment rows, and the draft's saved equipment is unchanged.</t>
+          <t>"4K Portable Projector" is not listed as an option in the second row's dropdown — only items not already chosen elsewhere are offered. Choosing a different item in the second row and clicking "Save draft" saves both rows successfully.</t>
         </is>
       </c>
     </row>
@@ -2256,11 +2291,11 @@
       </c>
       <c r="B2" s="13" t="inlineStr">
         <is>
-          <t>SPM-24-TC14</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="31" customHeight="1">
+          <t>SPM-24-TC13b</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="44.5" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
@@ -2268,11 +2303,11 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>The draft from TC09 has Event name, Type, Starts at and Ends at set. Expected attendance is still missing.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="44.5" customHeight="1">
+          <t>The draft from TC09 already has Starts at and Ends at saved. Note the total number of active items shown across the equipment dropdown (N).</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="58" customHeight="1">
       <c r="A4" s="12" t="inlineStr">
         <is>
           <t>Test Steps</t>
@@ -2281,12 +2316,11 @@
       <c r="B4" s="13" t="inlineStr">
         <is>
           <t>1. Open the draft's "Edit draft" page
-2. Enter 120 into Expected attendance
-3. Click "Submit request"</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="31" customHeight="1">
+2. Click "Add equipment" and pick a different, not-yet-chosen item in each row, N times in total, until every catalogue item has been used</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="17.5" customHeight="1">
       <c r="A5" s="12" t="inlineStr">
         <is>
           <t>Test Data</t>
@@ -2294,7 +2328,7 @@
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>Expected attendance: 120 (everything else already saved from TC09)</t>
+          <t>One row per catalogue item, no repeats</t>
         </is>
       </c>
     </row>
@@ -2306,7 +2340,7 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>The browser moves to the event's own page. Its status badge now reads "Submitted" instead of "Draft", and it no longer appears under "Drafts — not yet submitted" on "My events".</t>
+          <t>Once the last item is chosen, the "Add equipment" button becomes disabled and the text "Every catalogue item is already in your request." appears beneath it.</t>
         </is>
       </c>
     </row>
@@ -2415,11 +2449,11 @@
       </c>
       <c r="B2" s="13" t="inlineStr">
         <is>
-          <t>SPM-24-TC15</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="58" customHeight="1">
+          <t>SPM-24-TC14</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="31" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
@@ -2427,7 +2461,7 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>The seeded draft "Q1 Investor Update (rough idea)", owned by rachel.ng@meridianfina.com, has only a title and description — Type of event, Starts at, Ends at and Expected attendance are all still empty.</t>
+          <t>The draft from TC09 has Event name, Type, Starts at and Ends at set. Expected attendance is still missing.</t>
         </is>
       </c>
     </row>
@@ -2439,13 +2473,13 @@
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>1. Log in as rachel.ng@meridianfina.com / password123
-2. Open the draft's "Edit draft" page
-3. Without filling anything else in, click "Submit request"</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="17.5" customHeight="1">
+          <t>1. Open the draft's "Edit draft" page
+2. Enter 120 into Expected attendance
+3. Click "Submit request"</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="31" customHeight="1">
       <c r="A5" s="12" t="inlineStr">
         <is>
           <t>Test Data</t>
@@ -2453,11 +2487,11 @@
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>N/A — submitting the draft exactly as saved</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="58" customHeight="1">
+          <t>Expected attendance: 120 (everything else already saved from TC09)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="44.5" customHeight="1">
       <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
@@ -2465,7 +2499,7 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>The page does not move on. Messages appear at once under Type of event, Starts at, Ends at and Expected attendance, listing what's still needed; the draft is left exactly as it was, still showing the "Draft" badge.</t>
+          <t>The browser moves to the event's own page. Its status badge now reads "Submitted" instead of "Draft", and it no longer appears under "Drafts — not yet submitted" on "My events".</t>
         </is>
       </c>
     </row>
@@ -2574,11 +2608,11 @@
       </c>
       <c r="B2" s="13" t="inlineStr">
         <is>
-          <t>SPM-24-TC16</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="44.5" customHeight="1">
+          <t>SPM-24-TC15</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="58" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
@@ -2586,11 +2620,11 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>Seeded account rachel.ng@meridianfina.com owns the seeded draft "Q1 Investor Update (rough idea)" and the seeded, already-completed event "Meridian Compliance Training".</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="31" customHeight="1">
+          <t>The seeded draft "Q1 Investor Update (rough idea)", owned by rachel.ng@meridianfina.com, has only a title and description — Type of event, Starts at, Ends at and Expected attendance are all still empty.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="44.5" customHeight="1">
       <c r="A4" s="12" t="inlineStr">
         <is>
           <t>Test Steps</t>
@@ -2599,7 +2633,8 @@
       <c r="B4" s="13" t="inlineStr">
         <is>
           <t>1. Log in as rachel.ng@meridianfina.com / password123
-2. Open the "My events" page</t>
+2. Open the draft's "Edit draft" page
+3. Without filling anything else in, click "Submit request"</t>
         </is>
       </c>
     </row>
@@ -2611,11 +2646,11 @@
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>N/A — uses seeded data</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="44.5" customHeight="1">
+          <t>N/A — submitting the draft exactly as saved</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="58" customHeight="1">
       <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
@@ -2623,7 +2658,7 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>The draft appears only under "Drafts — not yet submitted". The "Submitted" section lists "Meridian Compliance Training" but not "Q1 Investor Update (rough idea)".</t>
+          <t>The page does not move on. Messages appear at once under Type of event, Starts at, Ends at and Expected attendance, listing what's still needed; the draft is left exactly as it was, still showing the "Draft" badge.</t>
         </is>
       </c>
     </row>
@@ -2732,11 +2767,11 @@
       </c>
       <c r="B2" s="13" t="inlineStr">
         <is>
-          <t>SPM-24-TC17</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="71.5" customHeight="1">
+          <t>SPM-24-TC16</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="44.5" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
@@ -2744,7 +2779,7 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>daniel.tan@connectsphere.com is a seeded Coordinator who owns no events of his own. rachel.ng@meridianfina.com owns the seeded draft "Q1 Investor Update (rough idea)". budi.santoso@nusantaratec.com owns the seeded, already-submitted event "Nusantara Developer Summit".</t>
+          <t>Seeded account rachel.ng@meridianfina.com owns the seeded draft "Q1 Investor Update (rough idea)" and the seeded, already-completed event "Meridian Compliance Training".</t>
         </is>
       </c>
     </row>
@@ -2756,8 +2791,8 @@
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>1. Log in as daniel.tan@connectsphere.com / password123
-2. Open the "All events" page</t>
+          <t>1. Log in as rachel.ng@meridianfina.com / password123
+2. Open the "My events" page</t>
         </is>
       </c>
     </row>
@@ -2781,7 +2816,7 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>"Nusantara Developer Summit" appears in the list. "Q1 Investor Update (rough idea)", or any other draft, does not appear anywhere on the page.</t>
+          <t>The draft appears only under "Drafts — not yet submitted". The "Submitted" section lists "Meridian Compliance Training" but not "Q1 Investor Update (rough idea)".</t>
         </is>
       </c>
     </row>
@@ -2892,19 +2927,177 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="17.5" customHeight="1">
+    <row r="2" ht="152.5" customHeight="1">
       <c r="A2" s="11" t="n">
         <v>1</v>
       </c>
       <c r="B2" s="11" t="inlineStr">
         <is>
-          <t>None raised</t>
+          <t>SPM-24-TC13 originally tested that selecting the same equipment item twice was rejected after the fact, with an error message. The picker was changed so a duplicate can no longer be selected in the first place (the already-chosen item is removed from the other rows' dropdowns), which is why TC13 now tests prevention instead of rejection, and TC13b was added for the 'every item already used' edge case. The server-side Zod rule that used to produce the rejection message is still in place as a safety net (src/lib/validation/events.ts) but is no longer reachable by clicking through the app, so it isn't covered by a manual test case here — only by the existing unit test in src/lib/__tests__/validation.test.ts.</t>
         </is>
       </c>
       <c r="C2" s="11" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C15"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
+  <cols>
+    <col width="24.77734375" customWidth="1" min="1" max="1"/>
+    <col width="56.77734375" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="n"/>
+    </row>
+    <row r="2" ht="17.5" customHeight="1">
+      <c r="A2" s="12" t="inlineStr">
+        <is>
+          <t>Test Case ID</t>
+        </is>
+      </c>
+      <c r="B2" s="13" t="inlineStr">
+        <is>
+          <t>SPM-24-TC17</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="71.5" customHeight="1">
+      <c r="A3" s="12" t="inlineStr">
+        <is>
+          <t>Pre-conditions</t>
+        </is>
+      </c>
+      <c r="B3" s="13" t="inlineStr">
+        <is>
+          <t>daniel.tan@connectsphere.com is a seeded Coordinator who owns no events of his own. rachel.ng@meridianfina.com owns the seeded draft "Q1 Investor Update (rough idea)". budi.santoso@nusantaratec.com owns the seeded, already-submitted event "Nusantara Developer Summit".</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="31" customHeight="1">
+      <c r="A4" s="12" t="inlineStr">
+        <is>
+          <t>Test Steps</t>
+        </is>
+      </c>
+      <c r="B4" s="13" t="inlineStr">
+        <is>
+          <t>1. Log in as daniel.tan@connectsphere.com / password123
+2. Open the "All events" page</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="17.5" customHeight="1">
+      <c r="A5" s="12" t="inlineStr">
+        <is>
+          <t>Test Data</t>
+        </is>
+      </c>
+      <c r="B5" s="13" t="inlineStr">
+        <is>
+          <t>N/A — uses seeded data</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="44.5" customHeight="1">
+      <c r="A6" s="12" t="inlineStr">
+        <is>
+          <t>Expected Result</t>
+        </is>
+      </c>
+      <c r="B6" s="13" t="inlineStr">
+        <is>
+          <t>"Nusantara Developer Summit" appears in the list. "Q1 Investor Update (rough idea)", or any other draft, does not appear anywhere on the page.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="17.5" customHeight="1">
+      <c r="A7" s="12" t="inlineStr">
+        <is>
+          <t>Created By</t>
+        </is>
+      </c>
+      <c r="B7" s="13" t="inlineStr">
+        <is>
+          <t>kchoongg</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="12" t="inlineStr">
+        <is>
+          <t>Creation Date</t>
+        </is>
+      </c>
+      <c r="B8" s="14" t="n">
+        <v>46281</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n"/>
+      <c r="C10" s="6" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>Actual Result</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>Pass/Fail/Not Executed/Blocked</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Remarks</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>Executed by</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>Date of Execution</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 

</xml_diff>